<commit_message>
fix: add EBO Store - Virar (site 1021) to SITE_MASTER
</commit_message>
<xml_diff>
--- a/Odoo_Ginesys_DC_TransferOut_Automation_V4_5_WorkDateFix/Master/Ginesys_Config.xlsx
+++ b/Odoo_Ginesys_DC_TransferOut_Automation_V4_5_WorkDateFix/Master/Ginesys_Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Test_API\Odoo_Ginesys_DC_TransferOut_Automation_V4_5_WorkDateFix\Master\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\odoo automation\Odoo_Ginesys_DC_TransferOut_Automation_V4_5_WorkDateFix\Master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ED174E1-D821-4B79-82BA-385B4793F098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1836D37-EA40-499A-95BE-7D3603FC761C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="FIELD_GUIDE" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">SITE_MASTER!$A$1:$G$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">SITE_MASTER!$A$1:$G$111</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="348">
   <si>
     <t>Purpose</t>
   </si>
@@ -1085,6 +1085,9 @@
   </si>
   <si>
     <t>TECHNO SPORTSWEAR PRIVATE LIMITED(WB), EBO Store - Chandan Nagar</t>
+  </si>
+  <si>
+    <t>TECHNO SPORTSWEAR PRIVATE LIMITED(MH), EBO Store - Virar</t>
   </si>
 </sst>
 </file>
@@ -1452,7 +1455,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
@@ -1470,7 +1473,7 @@
       <c r="G1" s="21"/>
       <c r="H1" s="21"/>
     </row>
-    <row r="3" spans="1:8" ht="27.4">
+    <row r="3" spans="1:8" ht="28">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1478,7 +1481,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="13.9">
+    <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
         <v>242</v>
       </c>
@@ -1486,7 +1489,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="27.4">
+    <row r="5" spans="1:8" ht="28">
       <c r="A5" s="1" t="s">
         <v>244</v>
       </c>
@@ -1494,7 +1497,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="27.4">
+    <row r="6" spans="1:8" ht="28">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -1502,7 +1505,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="13.9">
+    <row r="7" spans="1:8">
       <c r="A7" s="1" t="s">
         <v>2</v>
       </c>
@@ -1510,7 +1513,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="13.9">
+    <row r="8" spans="1:8">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1518,7 +1521,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="13.9">
+    <row r="9" spans="1:8">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
@@ -1526,7 +1529,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="27.4">
+    <row r="10" spans="1:8" ht="28">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
@@ -1534,7 +1537,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="13.9">
+    <row r="12" spans="1:8">
       <c r="A12" s="3" t="s">
         <v>6</v>
       </c>
@@ -1542,7 +1545,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="13.9">
+    <row r="13" spans="1:8">
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
@@ -1550,7 +1553,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="13.9">
+    <row r="14" spans="1:8">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
@@ -1558,7 +1561,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="13.9">
+    <row r="15" spans="1:8">
       <c r="A15" s="1" t="s">
         <v>253</v>
       </c>
@@ -1566,7 +1569,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="13.9">
+    <row r="16" spans="1:8">
       <c r="A16" s="1" t="s">
         <v>255</v>
       </c>
@@ -1585,10 +1588,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O8"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="2" width="17.125" customWidth="1"/>
+    <col min="2" max="2" width="17.08203125" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="34" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
@@ -1602,7 +1605,7 @@
     <col min="15" max="15" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="35.1" customHeight="1">
+    <row r="1" spans="1:15" ht="35.15" customHeight="1">
       <c r="A1" s="4" t="s">
         <v>10</v>
       </c>
@@ -1649,7 +1652,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="27">
+    <row r="2" spans="1:15" ht="28">
       <c r="A2" s="15" t="s">
         <v>23</v>
       </c>
@@ -1688,7 +1691,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="13.9">
+    <row r="4" spans="1:15">
       <c r="A4" s="22" t="s">
         <v>27</v>
       </c>
@@ -1707,7 +1710,7 @@
       <c r="N4" s="23"/>
       <c r="O4" s="23"/>
     </row>
-    <row r="5" spans="1:15" ht="13.9">
+    <row r="5" spans="1:15">
       <c r="A5" s="8" t="s">
         <v>10</v>
       </c>
@@ -1728,7 +1731,7 @@
       <c r="N5" s="24"/>
       <c r="O5" s="24"/>
     </row>
-    <row r="6" spans="1:15" ht="13.9">
+    <row r="6" spans="1:15">
       <c r="A6" s="8" t="s">
         <v>11</v>
       </c>
@@ -1749,7 +1752,7 @@
       <c r="N6" s="24"/>
       <c r="O6" s="24"/>
     </row>
-    <row r="7" spans="1:15" ht="13.9">
+    <row r="7" spans="1:15">
       <c r="A7" s="8" t="s">
         <v>29</v>
       </c>
@@ -1770,7 +1773,7 @@
       <c r="N7" s="24"/>
       <c r="O7" s="24"/>
     </row>
-    <row r="8" spans="1:15" ht="13.9">
+    <row r="8" spans="1:15">
       <c r="A8" s="8" t="s">
         <v>261</v>
       </c>
@@ -1813,20 +1816,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G200"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="105" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="65.625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.58203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="65.58203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="32.1" customHeight="1">
+    <row r="1" spans="1:7" ht="32.15" customHeight="1">
       <c r="A1" s="4" t="s">
         <v>31</v>
       </c>
@@ -1849,7 +1851,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:7" hidden="1">
+    <row r="2" spans="1:7">
       <c r="A2" s="5" t="s">
         <v>36</v>
       </c>
@@ -1870,7 +1872,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:7" hidden="1">
+    <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
         <v>38</v>
       </c>
@@ -1891,7 +1893,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:7" hidden="1">
+    <row r="4" spans="1:7">
       <c r="A4" s="5" t="s">
         <v>40</v>
       </c>
@@ -1912,7 +1914,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:7" hidden="1">
+    <row r="5" spans="1:7">
       <c r="A5" s="5" t="s">
         <v>42</v>
       </c>
@@ -1933,7 +1935,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:7" hidden="1">
+    <row r="6" spans="1:7">
       <c r="A6" s="5" t="s">
         <v>44</v>
       </c>
@@ -1954,7 +1956,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1">
+    <row r="7" spans="1:7">
       <c r="A7" s="5" t="s">
         <v>46</v>
       </c>
@@ -1975,7 +1977,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1">
+    <row r="8" spans="1:7">
       <c r="A8" s="5" t="s">
         <v>48</v>
       </c>
@@ -1996,7 +1998,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1">
+    <row r="9" spans="1:7">
       <c r="A9" s="5" t="s">
         <v>50</v>
       </c>
@@ -2017,7 +2019,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:7" hidden="1">
+    <row r="10" spans="1:7">
       <c r="A10" s="5" t="s">
         <v>52</v>
       </c>
@@ -2038,7 +2040,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1">
+    <row r="11" spans="1:7">
       <c r="A11" s="5" t="s">
         <v>54</v>
       </c>
@@ -2059,7 +2061,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:7" hidden="1">
+    <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
         <v>56</v>
       </c>
@@ -2080,7 +2082,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:7" hidden="1">
+    <row r="13" spans="1:7">
       <c r="A13" s="5" t="s">
         <v>58</v>
       </c>
@@ -2101,7 +2103,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1">
+    <row r="14" spans="1:7">
       <c r="A14" s="5" t="s">
         <v>60</v>
       </c>
@@ -2122,7 +2124,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1">
+    <row r="15" spans="1:7">
       <c r="A15" s="5" t="s">
         <v>62</v>
       </c>
@@ -2143,7 +2145,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1">
+    <row r="16" spans="1:7">
       <c r="A16" s="5" t="s">
         <v>64</v>
       </c>
@@ -2164,7 +2166,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:7" hidden="1">
+    <row r="17" spans="1:7">
       <c r="A17" s="5" t="s">
         <v>66</v>
       </c>
@@ -2185,7 +2187,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:7" hidden="1">
+    <row r="18" spans="1:7">
       <c r="A18" s="5" t="s">
         <v>68</v>
       </c>
@@ -2206,7 +2208,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:7" hidden="1">
+    <row r="19" spans="1:7">
       <c r="A19" s="5" t="s">
         <v>70</v>
       </c>
@@ -2227,7 +2229,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:7" hidden="1">
+    <row r="20" spans="1:7">
       <c r="A20" s="5" t="s">
         <v>72</v>
       </c>
@@ -2248,7 +2250,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:7" hidden="1">
+    <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
         <v>74</v>
       </c>
@@ -2269,7 +2271,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:7" hidden="1">
+    <row r="22" spans="1:7">
       <c r="A22" s="5" t="s">
         <v>76</v>
       </c>
@@ -2290,7 +2292,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:7" hidden="1">
+    <row r="23" spans="1:7">
       <c r="A23" s="5" t="s">
         <v>78</v>
       </c>
@@ -2311,7 +2313,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:7" hidden="1">
+    <row r="24" spans="1:7">
       <c r="A24" s="5" t="s">
         <v>80</v>
       </c>
@@ -2332,7 +2334,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:7" hidden="1">
+    <row r="25" spans="1:7">
       <c r="A25" s="5" t="s">
         <v>82</v>
       </c>
@@ -2353,7 +2355,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:7" hidden="1">
+    <row r="26" spans="1:7">
       <c r="A26" s="5" t="s">
         <v>84</v>
       </c>
@@ -2374,7 +2376,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:7" hidden="1">
+    <row r="27" spans="1:7">
       <c r="A27" s="5" t="s">
         <v>86</v>
       </c>
@@ -2395,7 +2397,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:7" hidden="1">
+    <row r="28" spans="1:7">
       <c r="A28" s="5" t="s">
         <v>88</v>
       </c>
@@ -2416,7 +2418,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:7" hidden="1">
+    <row r="29" spans="1:7">
       <c r="A29" s="5" t="s">
         <v>90</v>
       </c>
@@ -2437,7 +2439,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:7" hidden="1">
+    <row r="30" spans="1:7">
       <c r="A30" s="5" t="s">
         <v>92</v>
       </c>
@@ -2458,7 +2460,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:7" hidden="1">
+    <row r="31" spans="1:7">
       <c r="A31" s="5" t="s">
         <v>94</v>
       </c>
@@ -2479,7 +2481,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:7" hidden="1">
+    <row r="32" spans="1:7">
       <c r="A32" s="5" t="s">
         <v>96</v>
       </c>
@@ -2500,7 +2502,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:7" hidden="1">
+    <row r="33" spans="1:7">
       <c r="A33" s="5" t="s">
         <v>98</v>
       </c>
@@ -2521,7 +2523,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:7" hidden="1">
+    <row r="34" spans="1:7">
       <c r="A34" s="5" t="s">
         <v>100</v>
       </c>
@@ -2542,7 +2544,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:7" hidden="1">
+    <row r="35" spans="1:7">
       <c r="A35" s="5" t="s">
         <v>102</v>
       </c>
@@ -2563,7 +2565,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:7" hidden="1">
+    <row r="36" spans="1:7">
       <c r="A36" s="5" t="s">
         <v>104</v>
       </c>
@@ -2584,7 +2586,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:7" hidden="1">
+    <row r="37" spans="1:7">
       <c r="A37" s="5" t="s">
         <v>106</v>
       </c>
@@ -2605,7 +2607,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:7" hidden="1">
+    <row r="38" spans="1:7">
       <c r="A38" s="5" t="s">
         <v>108</v>
       </c>
@@ -2626,7 +2628,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:7" hidden="1">
+    <row r="39" spans="1:7">
       <c r="A39" s="5" t="s">
         <v>110</v>
       </c>
@@ -2647,7 +2649,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="1:7" hidden="1">
+    <row r="40" spans="1:7">
       <c r="A40" s="5" t="s">
         <v>112</v>
       </c>
@@ -2668,7 +2670,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="41" spans="1:7" hidden="1">
+    <row r="41" spans="1:7">
       <c r="A41" s="5" t="s">
         <v>114</v>
       </c>
@@ -2689,7 +2691,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="1:7" hidden="1">
+    <row r="42" spans="1:7">
       <c r="A42" s="5" t="s">
         <v>116</v>
       </c>
@@ -2710,7 +2712,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:7" hidden="1">
+    <row r="43" spans="1:7">
       <c r="A43" s="5" t="s">
         <v>118</v>
       </c>
@@ -2731,7 +2733,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:7" hidden="1">
+    <row r="44" spans="1:7">
       <c r="A44" s="5" t="s">
         <v>120</v>
       </c>
@@ -2752,7 +2754,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="45" spans="1:7" hidden="1">
+    <row r="45" spans="1:7">
       <c r="A45" s="5" t="s">
         <v>122</v>
       </c>
@@ -2773,7 +2775,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:7" hidden="1">
+    <row r="46" spans="1:7">
       <c r="A46" s="5" t="s">
         <v>124</v>
       </c>
@@ -2794,7 +2796,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="47" spans="1:7" hidden="1">
+    <row r="47" spans="1:7">
       <c r="A47" s="5" t="s">
         <v>126</v>
       </c>
@@ -2815,7 +2817,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="48" spans="1:7" hidden="1">
+    <row r="48" spans="1:7">
       <c r="A48" s="5" t="s">
         <v>128</v>
       </c>
@@ -2836,7 +2838,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:7" hidden="1">
+    <row r="49" spans="1:7">
       <c r="A49" s="5" t="s">
         <v>130</v>
       </c>
@@ -2857,7 +2859,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="50" spans="1:7" hidden="1">
+    <row r="50" spans="1:7">
       <c r="A50" s="5" t="s">
         <v>281</v>
       </c>
@@ -2878,7 +2880,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="51" spans="1:7" hidden="1">
+    <row r="51" spans="1:7">
       <c r="A51" s="5" t="s">
         <v>133</v>
       </c>
@@ -2899,7 +2901,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:7" hidden="1">
+    <row r="52" spans="1:7">
       <c r="A52" s="5" t="s">
         <v>135</v>
       </c>
@@ -2920,7 +2922,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:7" hidden="1">
+    <row r="53" spans="1:7">
       <c r="A53" s="5" t="s">
         <v>137</v>
       </c>
@@ -2941,7 +2943,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="54" spans="1:7" hidden="1">
+    <row r="54" spans="1:7">
       <c r="A54" s="5" t="s">
         <v>139</v>
       </c>
@@ -2962,7 +2964,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="55" spans="1:7" hidden="1">
+    <row r="55" spans="1:7">
       <c r="A55" s="5" t="s">
         <v>141</v>
       </c>
@@ -2983,7 +2985,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:7" hidden="1">
+    <row r="56" spans="1:7">
       <c r="A56" s="5" t="s">
         <v>143</v>
       </c>
@@ -3004,7 +3006,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="57" spans="1:7" hidden="1">
+    <row r="57" spans="1:7">
       <c r="A57" s="5" t="s">
         <v>145</v>
       </c>
@@ -3025,7 +3027,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="58" spans="1:7" hidden="1">
+    <row r="58" spans="1:7">
       <c r="A58" s="5" t="s">
         <v>147</v>
       </c>
@@ -3046,7 +3048,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:7" hidden="1">
+    <row r="59" spans="1:7">
       <c r="A59" s="5" t="s">
         <v>149</v>
       </c>
@@ -3067,7 +3069,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:7" hidden="1">
+    <row r="60" spans="1:7">
       <c r="A60" s="5" t="s">
         <v>151</v>
       </c>
@@ -3088,7 +3090,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="61" spans="1:7" hidden="1">
+    <row r="61" spans="1:7">
       <c r="A61" s="5" t="s">
         <v>153</v>
       </c>
@@ -3109,7 +3111,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="62" spans="1:7" hidden="1">
+    <row r="62" spans="1:7">
       <c r="A62" s="5" t="s">
         <v>155</v>
       </c>
@@ -3130,7 +3132,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="63" spans="1:7" hidden="1">
+    <row r="63" spans="1:7">
       <c r="A63" s="5" t="s">
         <v>157</v>
       </c>
@@ -3151,7 +3153,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="64" spans="1:7" hidden="1">
+    <row r="64" spans="1:7">
       <c r="A64" s="5" t="s">
         <v>159</v>
       </c>
@@ -3172,7 +3174,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="1:7" hidden="1">
+    <row r="65" spans="1:7">
       <c r="A65" s="5" t="s">
         <v>161</v>
       </c>
@@ -3193,7 +3195,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="66" spans="1:7" hidden="1">
+    <row r="66" spans="1:7">
       <c r="A66" s="5" t="s">
         <v>163</v>
       </c>
@@ -3214,7 +3216,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="67" spans="1:7" hidden="1">
+    <row r="67" spans="1:7">
       <c r="A67" s="5" t="s">
         <v>165</v>
       </c>
@@ -3235,7 +3237,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:7" hidden="1">
+    <row r="68" spans="1:7">
       <c r="A68" s="5" t="s">
         <v>167</v>
       </c>
@@ -3256,7 +3258,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="69" spans="1:7" hidden="1">
+    <row r="69" spans="1:7">
       <c r="A69" s="5" t="s">
         <v>169</v>
       </c>
@@ -3277,7 +3279,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="70" spans="1:7" hidden="1">
+    <row r="70" spans="1:7">
       <c r="A70" s="5" t="s">
         <v>170</v>
       </c>
@@ -3298,7 +3300,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="71" spans="1:7" hidden="1">
+    <row r="71" spans="1:7">
       <c r="A71" s="5" t="s">
         <v>159</v>
       </c>
@@ -3319,7 +3321,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:7" hidden="1">
+    <row r="72" spans="1:7">
       <c r="A72" s="5" t="s">
         <v>172</v>
       </c>
@@ -3340,7 +3342,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="73" spans="1:7" hidden="1">
+    <row r="73" spans="1:7">
       <c r="A73" s="5" t="s">
         <v>174</v>
       </c>
@@ -3361,7 +3363,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="74" spans="1:7" hidden="1">
+    <row r="74" spans="1:7">
       <c r="A74" s="5" t="s">
         <v>176</v>
       </c>
@@ -3382,7 +3384,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="75" spans="1:7" hidden="1">
+    <row r="75" spans="1:7">
       <c r="A75" t="s">
         <v>283</v>
       </c>
@@ -3403,7 +3405,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="76" spans="1:7" hidden="1">
+    <row r="76" spans="1:7">
       <c r="A76" s="5" t="s">
         <v>285</v>
       </c>
@@ -3424,7 +3426,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="77" spans="1:7" hidden="1">
+    <row r="77" spans="1:7">
       <c r="A77" s="5" t="s">
         <v>286</v>
       </c>
@@ -3445,7 +3447,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="78" spans="1:7" hidden="1">
+    <row r="78" spans="1:7">
       <c r="A78" s="5" t="s">
         <v>288</v>
       </c>
@@ -3466,7 +3468,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:7" hidden="1">
+    <row r="79" spans="1:7">
       <c r="A79" s="5" t="s">
         <v>289</v>
       </c>
@@ -3487,7 +3489,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="80" spans="1:7" hidden="1">
+    <row r="80" spans="1:7">
       <c r="A80" s="5" t="s">
         <v>291</v>
       </c>
@@ -3508,7 +3510,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:7" hidden="1">
+    <row r="81" spans="1:7">
       <c r="A81" s="5" t="s">
         <v>293</v>
       </c>
@@ -3529,7 +3531,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="82" spans="1:7" hidden="1">
+    <row r="82" spans="1:7">
       <c r="A82" s="5" t="s">
         <v>294</v>
       </c>
@@ -3550,7 +3552,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="83" spans="1:7" hidden="1">
+    <row r="83" spans="1:7">
       <c r="A83" s="5" t="s">
         <v>295</v>
       </c>
@@ -3571,7 +3573,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="84" spans="1:7" hidden="1">
+    <row r="84" spans="1:7">
       <c r="A84" s="5" t="s">
         <v>297</v>
       </c>
@@ -3592,7 +3594,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="85" spans="1:7" hidden="1">
+    <row r="85" spans="1:7">
       <c r="A85" s="5" t="s">
         <v>299</v>
       </c>
@@ -3613,7 +3615,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="86" spans="1:7" hidden="1">
+    <row r="86" spans="1:7">
       <c r="A86" s="5" t="s">
         <v>300</v>
       </c>
@@ -3634,7 +3636,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="87" spans="1:7" hidden="1">
+    <row r="87" spans="1:7">
       <c r="A87" s="5" t="s">
         <v>302</v>
       </c>
@@ -3655,7 +3657,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:7" hidden="1">
+    <row r="88" spans="1:7">
       <c r="A88" s="5" t="s">
         <v>303</v>
       </c>
@@ -3676,7 +3678,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="89" spans="1:7" hidden="1">
+    <row r="89" spans="1:7">
       <c r="A89" s="5" t="s">
         <v>304</v>
       </c>
@@ -3697,7 +3699,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="90" spans="1:7" hidden="1">
+    <row r="90" spans="1:7">
       <c r="A90" s="5" t="s">
         <v>305</v>
       </c>
@@ -3718,7 +3720,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="91" spans="1:7" hidden="1">
+    <row r="91" spans="1:7">
       <c r="A91" s="5" t="s">
         <v>306</v>
       </c>
@@ -3739,7 +3741,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="92" spans="1:7" hidden="1">
+    <row r="92" spans="1:7">
       <c r="A92" s="5" t="s">
         <v>307</v>
       </c>
@@ -3760,7 +3762,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="93" spans="1:7" hidden="1">
+    <row r="93" spans="1:7">
       <c r="A93" s="5" t="s">
         <v>308</v>
       </c>
@@ -3781,7 +3783,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="94" spans="1:7" hidden="1">
+    <row r="94" spans="1:7">
       <c r="A94" s="5" t="s">
         <v>310</v>
       </c>
@@ -3802,7 +3804,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="95" spans="1:7" hidden="1">
+    <row r="95" spans="1:7">
       <c r="A95" s="5" t="s">
         <v>313</v>
       </c>
@@ -3844,7 +3846,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="97" spans="1:7" hidden="1">
+    <row r="97" spans="1:7">
       <c r="A97" s="5" t="s">
         <v>318</v>
       </c>
@@ -3865,7 +3867,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="98" spans="1:7" hidden="1">
+    <row r="98" spans="1:7">
       <c r="A98" s="5" t="s">
         <v>320</v>
       </c>
@@ -3886,7 +3888,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="99" spans="1:7" hidden="1">
+    <row r="99" spans="1:7">
       <c r="A99" s="5" t="s">
         <v>322</v>
       </c>
@@ -3907,7 +3909,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="100" spans="1:7" hidden="1">
+    <row r="100" spans="1:7">
       <c r="A100" s="5" t="s">
         <v>323</v>
       </c>
@@ -3928,7 +3930,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="101" spans="1:7" hidden="1">
+    <row r="101" spans="1:7">
       <c r="A101" s="5" t="s">
         <v>324</v>
       </c>
@@ -3949,7 +3951,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="102" spans="1:7" hidden="1">
+    <row r="102" spans="1:7">
       <c r="A102" s="5" t="s">
         <v>337</v>
       </c>
@@ -3970,7 +3972,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="103" spans="1:7" hidden="1">
+    <row r="103" spans="1:7">
       <c r="A103" s="5" t="s">
         <v>338</v>
       </c>
@@ -3991,7 +3993,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="104" spans="1:7" hidden="1">
+    <row r="104" spans="1:7">
       <c r="A104" s="5" t="s">
         <v>339</v>
       </c>
@@ -4012,7 +4014,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="105" spans="1:7" hidden="1">
+    <row r="105" spans="1:7">
       <c r="A105" s="5" t="s">
         <v>340</v>
       </c>
@@ -4033,7 +4035,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="106" spans="1:7" hidden="1">
+    <row r="106" spans="1:7">
       <c r="A106" s="5" t="s">
         <v>341</v>
       </c>
@@ -4054,7 +4056,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="107" spans="1:7" hidden="1">
+    <row r="107" spans="1:7">
       <c r="A107" s="5" t="s">
         <v>342</v>
       </c>
@@ -4075,7 +4077,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="108" spans="1:7" hidden="1">
+    <row r="108" spans="1:7">
       <c r="A108" s="5" t="s">
         <v>343</v>
       </c>
@@ -4096,7 +4098,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="109" spans="1:7" hidden="1">
+    <row r="109" spans="1:7">
       <c r="A109" s="5" t="s">
         <v>344</v>
       </c>
@@ -4117,7 +4119,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="110" spans="1:7" hidden="1">
+    <row r="110" spans="1:7">
       <c r="A110" s="5" t="s">
         <v>345</v>
       </c>
@@ -4160,13 +4162,25 @@
       </c>
     </row>
     <row r="112" spans="1:7">
-      <c r="A112" s="5"/>
-      <c r="B112" s="5"/>
-      <c r="C112" s="5"/>
-      <c r="D112" s="7"/>
+      <c r="A112" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="B112" s="5">
+        <v>1021</v>
+      </c>
+      <c r="C112" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="D112" s="7" t="s">
+        <v>314</v>
+      </c>
       <c r="E112" s="7"/>
-      <c r="F112" s="5"/>
-      <c r="G112" s="7"/>
+      <c r="F112" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G112" s="7" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="113" spans="1:7">
       <c r="A113" s="5"/>
@@ -4961,13 +4975,6 @@
       <c r="G200" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G110" xr:uid="{00000000-0001-0000-0200-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="TECHNO SPORTSWEAR PRIVATE LIMITED(WB), Chandan Nagar (EBO Store - Chandan Nagar)"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <dataValidations count="1">
     <dataValidation type="list" sqref="F2:F200" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"true,false"</formula1>
@@ -4981,7 +4988,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:W6"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -5274,7 +5281,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F500"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="3" width="16" customWidth="1"/>
@@ -9323,7 +9330,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -9331,7 +9338,7 @@
     <col min="4" max="4" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="13.9">
+    <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
         <v>6</v>
       </c>
@@ -9359,7 +9366,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="27">
+    <row r="3" spans="1:4" ht="28">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -9387,7 +9394,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="27">
+    <row r="5" spans="1:4" ht="28">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -9485,7 +9492,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="27">
+    <row r="12" spans="1:4" ht="28">
       <c r="A12" s="2" t="s">
         <v>268</v>
       </c>
@@ -9499,7 +9506,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="27">
+    <row r="13" spans="1:4" ht="28">
       <c r="A13" s="2" t="s">
         <v>268</v>
       </c>
@@ -9513,7 +9520,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="27">
+    <row r="14" spans="1:4" ht="28">
       <c r="A14" s="2" t="s">
         <v>268</v>
       </c>
@@ -9527,7 +9534,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="27">
+    <row r="15" spans="1:4" ht="28">
       <c r="A15" s="2" t="s">
         <v>268</v>
       </c>
@@ -9541,7 +9548,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="27">
+    <row r="16" spans="1:4" ht="28">
       <c r="A16" s="2" t="s">
         <v>268</v>
       </c>
@@ -9555,7 +9562,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="27">
+    <row r="17" spans="1:4" ht="28">
       <c r="A17" s="2" t="s">
         <v>268</v>
       </c>
@@ -9569,7 +9576,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="27">
+    <row r="18" spans="1:4" ht="28">
       <c r="A18" s="2" t="s">
         <v>268</v>
       </c>
@@ -9583,7 +9590,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="27">
+    <row r="19" spans="1:4" ht="28">
       <c r="A19" s="2" t="s">
         <v>268</v>
       </c>
@@ -9597,7 +9604,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="27">
+    <row r="20" spans="1:4" ht="28">
       <c r="A20" s="2" t="s">
         <v>268</v>
       </c>
@@ -9611,7 +9618,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="27">
+    <row r="21" spans="1:4" ht="28">
       <c r="A21" s="2" t="s">
         <v>280</v>
       </c>

</xml_diff>